<commit_message>
abstract for stan con
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCED13E-6D3D-46A7-83BE-6684B945CA16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A677EE9F-EBC3-4A23-8CCC-211F63DC43AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB08" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3788" uniqueCount="1246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3789" uniqueCount="1248">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4031,6 +4031,14 @@
   </si>
   <si>
     <t>MeasuredOn</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tip missing, narrow rings, can't see clearly</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mao</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4080,7 +4088,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4092,6 +4100,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4434,8 +4443,17 @@
       <c r="C4" t="s">
         <v>115</v>
       </c>
+      <c r="D4" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E4" s="5">
+        <v>46148</v>
+      </c>
+      <c r="F4">
+        <v>141</v>
+      </c>
       <c r="G4" t="s">
-        <v>1242</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -4447,6 +4465,9 @@
       </c>
       <c r="C5" t="s">
         <v>115</v>
+      </c>
+      <c r="F5">
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
keep record of core measurement
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A677EE9F-EBC3-4A23-8CCC-211F63DC43AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDE57C7-FA32-4EF0-BF13-0C78B1D3EA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,6 +25,7 @@
     <sheet name="TO04" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3789" uniqueCount="1248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3800" uniqueCount="1251">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4039,6 +4040,18 @@
   </si>
   <si>
     <t>Mao</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>can't measure the whole thing</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tip missing and can't measure the whole thing</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>there are some 'false ring'</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4421,6 +4434,12 @@
       <c r="C2" t="s">
         <v>115</v>
       </c>
+      <c r="D2" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E2" s="5">
+        <v>46148</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -4432,6 +4451,12 @@
       <c r="C3" t="s">
         <v>115</v>
       </c>
+      <c r="D3" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E3" s="5">
+        <v>46148</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -4466,6 +4491,12 @@
       <c r="C5" t="s">
         <v>115</v>
       </c>
+      <c r="D5" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E5" s="5">
+        <v>46148</v>
+      </c>
       <c r="F5">
         <v>150</v>
       </c>
@@ -4480,6 +4511,18 @@
       <c r="C6" t="s">
         <v>115</v>
       </c>
+      <c r="D6" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E6" s="5">
+        <v>46149</v>
+      </c>
+      <c r="F6">
+        <v>65</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1248</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -4491,6 +4534,18 @@
       <c r="C7" t="s">
         <v>115</v>
       </c>
+      <c r="D7" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E7" s="5">
+        <v>46149</v>
+      </c>
+      <c r="F7">
+        <v>112</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1248</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -4502,6 +4557,18 @@
       <c r="C8" t="s">
         <v>116</v>
       </c>
+      <c r="D8" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E8" s="5">
+        <v>46149</v>
+      </c>
+      <c r="F8">
+        <v>99</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1249</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -4512,6 +4579,18 @@
       </c>
       <c r="C9" t="s">
         <v>116</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E9" s="5">
+        <v>46149</v>
+      </c>
+      <c r="F9">
+        <v>199</v>
+      </c>
+      <c r="G9" t="s">
+        <v>1250</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated core measurement record
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F353E26-51C5-461A-A907-F7010018CCCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E48174-6F64-42E1-A394-AF4A23EDDB61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3801" uniqueCount="1251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3807" uniqueCount="1251">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4636,6 +4636,15 @@
       <c r="C12" t="s">
         <v>117</v>
       </c>
+      <c r="D12" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E12" s="5">
+        <v>46152</v>
+      </c>
+      <c r="F12">
+        <v>130</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -4647,6 +4656,15 @@
       <c r="C13" t="s">
         <v>117</v>
       </c>
+      <c r="D13" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E13" s="5">
+        <v>46152</v>
+      </c>
+      <c r="F13">
+        <v>130</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -4658,6 +4676,15 @@
       <c r="C14" t="s">
         <v>117</v>
       </c>
+      <c r="D14" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E14" s="5">
+        <v>46152</v>
+      </c>
+      <c r="F14">
+        <v>130</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -4669,6 +4696,15 @@
       <c r="C15" t="s">
         <v>117</v>
       </c>
+      <c r="D15" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E15" s="5">
+        <v>46152</v>
+      </c>
+      <c r="F15">
+        <v>130</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -4680,8 +4716,17 @@
       <c r="C16" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E16" s="5">
+        <v>46152</v>
+      </c>
+      <c r="F16">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -4691,8 +4736,17 @@
       <c r="C17" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E17" s="5">
+        <v>46152</v>
+      </c>
+      <c r="F17">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -4703,7 +4757,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -4714,7 +4768,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -4725,7 +4779,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -4736,7 +4790,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>3</v>
       </c>
@@ -4747,7 +4801,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>3</v>
       </c>
@@ -4758,7 +4812,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>3</v>
       </c>
@@ -4769,7 +4823,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -4780,7 +4834,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>3</v>
       </c>
@@ -4791,7 +4845,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>3</v>
       </c>
@@ -4802,7 +4856,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>3</v>
       </c>
@@ -4813,7 +4867,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>3</v>
       </c>
@@ -4824,7 +4878,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>3</v>
       </c>
@@ -4835,7 +4889,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>3</v>
       </c>
@@ -4846,7 +4900,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
update the records for core measurements
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E48174-6F64-42E1-A394-AF4A23EDDB61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3144AE1A-9FAC-4134-8B18-29BF59A1239D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3807" uniqueCount="1251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3809" uniqueCount="1253">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4051,6 +4051,14 @@
   </si>
   <si>
     <t>there are some 'false ring'</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>black circles 125-126</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>86 can't see clearly</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4726,7 +4734,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -4746,7 +4754,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -4756,8 +4764,11 @@
       <c r="C18" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F18">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -4767,8 +4778,11 @@
       <c r="C19" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F19">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -4778,8 +4792,11 @@
       <c r="C20" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F20">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -4789,8 +4806,11 @@
       <c r="C21" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F21">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>3</v>
       </c>
@@ -4800,8 +4820,11 @@
       <c r="C22" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F22">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>3</v>
       </c>
@@ -4811,8 +4834,11 @@
       <c r="C23" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F23">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>3</v>
       </c>
@@ -4822,8 +4848,11 @@
       <c r="C24" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F24">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -4833,8 +4862,11 @@
       <c r="C25" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>3</v>
       </c>
@@ -4844,8 +4876,11 @@
       <c r="C26" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F26">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>3</v>
       </c>
@@ -4855,8 +4890,11 @@
       <c r="C27" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F27">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>3</v>
       </c>
@@ -4866,8 +4904,14 @@
       <c r="C28" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F28">
+        <v>130</v>
+      </c>
+      <c r="G28" t="s">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>3</v>
       </c>
@@ -4877,8 +4921,11 @@
       <c r="C29" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F29">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>3</v>
       </c>
@@ -4888,8 +4935,11 @@
       <c r="C30" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F30">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>3</v>
       </c>
@@ -4899,8 +4949,11 @@
       <c r="C31" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F31">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -4910,8 +4963,11 @@
       <c r="C32" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F32">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>3</v>
       </c>
@@ -4921,8 +4977,11 @@
       <c r="C33" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F33">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>3</v>
       </c>
@@ -4932,8 +4991,11 @@
       <c r="C34" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F34">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>3</v>
       </c>
@@ -4944,7 +5006,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>3</v>
       </c>
@@ -4954,8 +5016,14 @@
       <c r="C36" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F36">
+        <v>87</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1252</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>3</v>
       </c>
@@ -4965,8 +5033,11 @@
       <c r="C37" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F37">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -4976,8 +5047,11 @@
       <c r="C38" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F38">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -4987,8 +5061,11 @@
       <c r="C39" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F39">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -4998,8 +5075,11 @@
       <c r="C40" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F40">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -5010,7 +5090,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -5021,7 +5101,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -5032,7 +5112,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -5043,7 +5123,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -5054,7 +5134,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -5065,7 +5145,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -5076,7 +5156,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
updates the measurement record
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CFEB9F5-CE26-4290-814A-33C7D7884BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9A9292-7D5F-4263-9759-322D35DDF96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB08" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="TO04" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3812" uniqueCount="1256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3816" uniqueCount="1260">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4071,6 +4072,22 @@
   </si>
   <si>
     <t>unclear</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ring 12,13 unclear</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ring 9 uncertain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ring 79, 94</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>need to check the core</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -5209,7 +5226,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -5223,7 +5240,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -5237,7 +5254,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -5251,7 +5268,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -5265,7 +5282,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -5275,8 +5292,11 @@
       <c r="C53" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F53">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -5286,8 +5306,14 @@
       <c r="C54" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F54">
+        <v>130</v>
+      </c>
+      <c r="G54" t="s">
+        <v>1256</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -5297,8 +5323,11 @@
       <c r="C55" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F55">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>3</v>
       </c>
@@ -5308,8 +5337,11 @@
       <c r="C56" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F56">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>3</v>
       </c>
@@ -5319,8 +5351,14 @@
       <c r="C57" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F57">
+        <v>130</v>
+      </c>
+      <c r="G57" t="s">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>3</v>
       </c>
@@ -5330,8 +5368,11 @@
       <c r="C58" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F58">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>3</v>
       </c>
@@ -5341,8 +5382,11 @@
       <c r="C59" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F59">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>3</v>
       </c>
@@ -5352,8 +5396,11 @@
       <c r="C60" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F60">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>3</v>
       </c>
@@ -5363,8 +5410,11 @@
       <c r="C61" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F61">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>3</v>
       </c>
@@ -5374,8 +5424,11 @@
       <c r="C62" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F62">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>3</v>
       </c>
@@ -5385,8 +5438,11 @@
       <c r="C63" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F63">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>3</v>
       </c>
@@ -5396,8 +5452,14 @@
       <c r="C64" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F64">
+        <v>123</v>
+      </c>
+      <c r="G64" t="s">
+        <v>1258</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>3</v>
       </c>
@@ -5407,8 +5469,11 @@
       <c r="C65" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F65">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>3</v>
       </c>
@@ -5418,8 +5483,11 @@
       <c r="C66" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F66">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>3</v>
       </c>
@@ -5429,8 +5497,11 @@
       <c r="C67" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F67">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>3</v>
       </c>
@@ -5440,8 +5511,11 @@
       <c r="C68" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="G68" t="s">
+        <v>1259</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>3</v>
       </c>
@@ -5451,8 +5525,11 @@
       <c r="C69" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="F69">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>3</v>
       </c>
@@ -5463,7 +5540,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>3</v>
       </c>
@@ -5474,7 +5551,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>3</v>
       </c>
@@ -5485,7 +5562,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>3</v>
       </c>
@@ -5496,7 +5573,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>3</v>
       </c>
@@ -5507,7 +5584,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>3</v>
       </c>
@@ -5518,7 +5595,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>3</v>
       </c>
@@ -5529,7 +5606,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>3</v>
       </c>
@@ -5540,7 +5617,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>3</v>
       </c>
@@ -5551,7 +5628,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>3</v>
       </c>
@@ -5562,7 +5639,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
updated the measurement record
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9A9292-7D5F-4263-9759-322D35DDF96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E982A73E-8DF2-42E1-982A-C78DB6F451AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB08" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,6 @@
     <sheet name="TO04" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3816" uniqueCount="1260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3817" uniqueCount="1261">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4088,6 +4087,10 @@
   </si>
   <si>
     <t>need to check the core</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0-1 30-31 ring</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -5539,6 +5542,9 @@
       <c r="C70" t="s">
         <v>119</v>
       </c>
+      <c r="F70">
+        <v>130</v>
+      </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
@@ -5550,6 +5556,9 @@
       <c r="C71" t="s">
         <v>119</v>
       </c>
+      <c r="F71">
+        <v>130</v>
+      </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
@@ -5561,6 +5570,9 @@
       <c r="C72" t="s">
         <v>119</v>
       </c>
+      <c r="F72">
+        <v>130</v>
+      </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
@@ -5572,6 +5584,9 @@
       <c r="C73" t="s">
         <v>119</v>
       </c>
+      <c r="F73">
+        <v>130</v>
+      </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
@@ -5583,6 +5598,9 @@
       <c r="C74" t="s">
         <v>119</v>
       </c>
+      <c r="F74">
+        <v>130</v>
+      </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
@@ -5593,6 +5611,12 @@
       </c>
       <c r="C75" t="s">
         <v>119</v>
+      </c>
+      <c r="F75">
+        <v>130</v>
+      </c>
+      <c r="G75" t="s">
+        <v>1260</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated the core measurement record
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F496D8-AE64-45DD-BEF7-73EF33B54FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612CED0A-C85C-4ED8-AC05-DF42BC889177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3921" uniqueCount="1256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4016" uniqueCount="1256">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4818,6 +4818,9 @@
       <c r="C18" t="s">
         <v>117</v>
       </c>
+      <c r="D18" t="s">
+        <v>1246</v>
+      </c>
       <c r="F18">
         <v>130</v>
       </c>
@@ -4835,6 +4838,9 @@
       <c r="C19" t="s">
         <v>117</v>
       </c>
+      <c r="D19" t="s">
+        <v>1246</v>
+      </c>
       <c r="F19">
         <v>130</v>
       </c>
@@ -4852,6 +4858,9 @@
       <c r="C20" t="s">
         <v>117</v>
       </c>
+      <c r="D20" t="s">
+        <v>1246</v>
+      </c>
       <c r="F20">
         <v>130</v>
       </c>
@@ -4869,6 +4878,9 @@
       <c r="C21" t="s">
         <v>117</v>
       </c>
+      <c r="D21" t="s">
+        <v>1246</v>
+      </c>
       <c r="F21">
         <v>130</v>
       </c>
@@ -4886,6 +4898,9 @@
       <c r="C22" t="s">
         <v>117</v>
       </c>
+      <c r="D22" t="s">
+        <v>1246</v>
+      </c>
       <c r="F22">
         <v>130</v>
       </c>
@@ -4903,6 +4918,9 @@
       <c r="C23" t="s">
         <v>117</v>
       </c>
+      <c r="D23" t="s">
+        <v>1246</v>
+      </c>
       <c r="F23">
         <v>130</v>
       </c>
@@ -4920,6 +4938,9 @@
       <c r="C24" t="s">
         <v>117</v>
       </c>
+      <c r="D24" t="s">
+        <v>1246</v>
+      </c>
       <c r="F24">
         <v>130</v>
       </c>
@@ -4937,6 +4958,9 @@
       <c r="C25" t="s">
         <v>117</v>
       </c>
+      <c r="D25" t="s">
+        <v>1246</v>
+      </c>
       <c r="F25">
         <v>130</v>
       </c>
@@ -4954,6 +4978,9 @@
       <c r="C26" t="s">
         <v>117</v>
       </c>
+      <c r="D26" t="s">
+        <v>1246</v>
+      </c>
       <c r="F26">
         <v>130</v>
       </c>
@@ -4971,6 +4998,9 @@
       <c r="C27" t="s">
         <v>117</v>
       </c>
+      <c r="D27" t="s">
+        <v>1246</v>
+      </c>
       <c r="F27">
         <v>130</v>
       </c>
@@ -4988,6 +5018,9 @@
       <c r="C28" t="s">
         <v>117</v>
       </c>
+      <c r="D28" t="s">
+        <v>1246</v>
+      </c>
       <c r="F28">
         <v>130</v>
       </c>
@@ -5008,6 +5041,9 @@
       <c r="C29" t="s">
         <v>117</v>
       </c>
+      <c r="D29" t="s">
+        <v>1246</v>
+      </c>
       <c r="F29">
         <v>130</v>
       </c>
@@ -5025,6 +5061,9 @@
       <c r="C30" t="s">
         <v>117</v>
       </c>
+      <c r="D30" t="s">
+        <v>1246</v>
+      </c>
       <c r="F30">
         <v>130</v>
       </c>
@@ -5042,6 +5081,9 @@
       <c r="C31" t="s">
         <v>117</v>
       </c>
+      <c r="D31" t="s">
+        <v>1246</v>
+      </c>
       <c r="F31">
         <v>130</v>
       </c>
@@ -5059,6 +5101,9 @@
       <c r="C32" t="s">
         <v>117</v>
       </c>
+      <c r="D32" t="s">
+        <v>1246</v>
+      </c>
       <c r="F32">
         <v>130</v>
       </c>
@@ -5076,6 +5121,9 @@
       <c r="C33" t="s">
         <v>117</v>
       </c>
+      <c r="D33" t="s">
+        <v>1246</v>
+      </c>
       <c r="F33">
         <v>130</v>
       </c>
@@ -5093,6 +5141,9 @@
       <c r="C34" t="s">
         <v>117</v>
       </c>
+      <c r="D34" t="s">
+        <v>1246</v>
+      </c>
       <c r="F34">
         <v>130</v>
       </c>
@@ -5110,6 +5161,9 @@
       <c r="C35" t="s">
         <v>117</v>
       </c>
+      <c r="D35" t="s">
+        <v>1246</v>
+      </c>
       <c r="H35" t="s">
         <v>1255</v>
       </c>
@@ -5124,6 +5178,9 @@
       <c r="C36" t="s">
         <v>117</v>
       </c>
+      <c r="D36" t="s">
+        <v>1246</v>
+      </c>
       <c r="F36">
         <v>87</v>
       </c>
@@ -5141,6 +5198,9 @@
       <c r="C37" t="s">
         <v>118</v>
       </c>
+      <c r="D37" t="s">
+        <v>1246</v>
+      </c>
       <c r="F37">
         <v>130</v>
       </c>
@@ -5158,6 +5218,9 @@
       <c r="C38" t="s">
         <v>118</v>
       </c>
+      <c r="D38" t="s">
+        <v>1246</v>
+      </c>
       <c r="F38">
         <v>137</v>
       </c>
@@ -5175,6 +5238,9 @@
       <c r="C39" t="s">
         <v>118</v>
       </c>
+      <c r="D39" t="s">
+        <v>1246</v>
+      </c>
       <c r="F39">
         <v>63</v>
       </c>
@@ -5192,6 +5258,9 @@
       <c r="C40" t="s">
         <v>118</v>
       </c>
+      <c r="D40" t="s">
+        <v>1246</v>
+      </c>
       <c r="F40">
         <v>68</v>
       </c>
@@ -5209,6 +5278,9 @@
       <c r="C41" t="s">
         <v>118</v>
       </c>
+      <c r="D41" t="s">
+        <v>1246</v>
+      </c>
       <c r="F41">
         <v>130</v>
       </c>
@@ -5226,6 +5298,9 @@
       <c r="C42" t="s">
         <v>118</v>
       </c>
+      <c r="D42" t="s">
+        <v>1246</v>
+      </c>
       <c r="F42">
         <v>130</v>
       </c>
@@ -5243,6 +5318,9 @@
       <c r="C43" t="s">
         <v>118</v>
       </c>
+      <c r="D43" t="s">
+        <v>1246</v>
+      </c>
       <c r="F43">
         <v>77</v>
       </c>
@@ -5260,6 +5338,9 @@
       <c r="C44" t="s">
         <v>118</v>
       </c>
+      <c r="D44" t="s">
+        <v>1246</v>
+      </c>
       <c r="F44">
         <v>81</v>
       </c>
@@ -5277,6 +5358,9 @@
       <c r="C45" t="s">
         <v>118</v>
       </c>
+      <c r="D45" t="s">
+        <v>1246</v>
+      </c>
       <c r="F45">
         <v>130</v>
       </c>
@@ -5294,6 +5378,9 @@
       <c r="C46" t="s">
         <v>118</v>
       </c>
+      <c r="D46" t="s">
+        <v>1246</v>
+      </c>
       <c r="G46" t="s">
         <v>1253</v>
       </c>
@@ -5311,6 +5398,9 @@
       <c r="C47" t="s">
         <v>118</v>
       </c>
+      <c r="D47" t="s">
+        <v>1246</v>
+      </c>
       <c r="F47">
         <v>130</v>
       </c>
@@ -5328,6 +5418,9 @@
       <c r="C48" t="s">
         <v>118</v>
       </c>
+      <c r="D48" t="s">
+        <v>1246</v>
+      </c>
       <c r="F48">
         <v>130</v>
       </c>
@@ -5345,6 +5438,9 @@
       <c r="C49" t="s">
         <v>118</v>
       </c>
+      <c r="D49" t="s">
+        <v>1246</v>
+      </c>
       <c r="F49">
         <v>130</v>
       </c>
@@ -5362,6 +5458,9 @@
       <c r="C50" t="s">
         <v>118</v>
       </c>
+      <c r="D50" t="s">
+        <v>1246</v>
+      </c>
       <c r="F50">
         <v>130</v>
       </c>
@@ -5379,6 +5478,9 @@
       <c r="C51" t="s">
         <v>118</v>
       </c>
+      <c r="D51" t="s">
+        <v>1246</v>
+      </c>
       <c r="F51">
         <v>130</v>
       </c>
@@ -5396,6 +5498,9 @@
       <c r="C52" t="s">
         <v>118</v>
       </c>
+      <c r="D52" t="s">
+        <v>1246</v>
+      </c>
       <c r="F52">
         <v>130</v>
       </c>
@@ -5413,6 +5518,9 @@
       <c r="C53" t="s">
         <v>118</v>
       </c>
+      <c r="D53" t="s">
+        <v>1246</v>
+      </c>
       <c r="F53">
         <v>130</v>
       </c>
@@ -5430,6 +5538,9 @@
       <c r="C54" t="s">
         <v>118</v>
       </c>
+      <c r="D54" t="s">
+        <v>1246</v>
+      </c>
       <c r="F54">
         <v>130</v>
       </c>
@@ -5447,6 +5558,9 @@
       <c r="C55" t="s">
         <v>118</v>
       </c>
+      <c r="D55" t="s">
+        <v>1246</v>
+      </c>
       <c r="F55">
         <v>130</v>
       </c>
@@ -5464,6 +5578,9 @@
       <c r="C56" t="s">
         <v>118</v>
       </c>
+      <c r="D56" t="s">
+        <v>1246</v>
+      </c>
       <c r="F56">
         <v>130</v>
       </c>
@@ -5481,6 +5598,9 @@
       <c r="C57" t="s">
         <v>118</v>
       </c>
+      <c r="D57" t="s">
+        <v>1246</v>
+      </c>
       <c r="F57">
         <v>130</v>
       </c>
@@ -5498,6 +5618,9 @@
       <c r="C58" t="s">
         <v>118</v>
       </c>
+      <c r="D58" t="s">
+        <v>1246</v>
+      </c>
       <c r="F58">
         <v>130</v>
       </c>
@@ -5515,6 +5638,9 @@
       <c r="C59" t="s">
         <v>118</v>
       </c>
+      <c r="D59" t="s">
+        <v>1246</v>
+      </c>
       <c r="F59">
         <v>130</v>
       </c>
@@ -5532,6 +5658,9 @@
       <c r="C60" t="s">
         <v>118</v>
       </c>
+      <c r="D60" t="s">
+        <v>1246</v>
+      </c>
       <c r="F60">
         <v>130</v>
       </c>
@@ -5549,6 +5678,9 @@
       <c r="C61" t="s">
         <v>118</v>
       </c>
+      <c r="D61" t="s">
+        <v>1246</v>
+      </c>
       <c r="F61">
         <v>130</v>
       </c>
@@ -5566,6 +5698,9 @@
       <c r="C62" t="s">
         <v>118</v>
       </c>
+      <c r="D62" t="s">
+        <v>1246</v>
+      </c>
       <c r="F62">
         <v>130</v>
       </c>
@@ -5583,6 +5718,9 @@
       <c r="C63" t="s">
         <v>118</v>
       </c>
+      <c r="D63" t="s">
+        <v>1246</v>
+      </c>
       <c r="F63">
         <v>117</v>
       </c>
@@ -5600,6 +5738,9 @@
       <c r="C64" t="s">
         <v>118</v>
       </c>
+      <c r="D64" t="s">
+        <v>1246</v>
+      </c>
       <c r="F64">
         <v>123</v>
       </c>
@@ -5620,6 +5761,9 @@
       <c r="C65" t="s">
         <v>118</v>
       </c>
+      <c r="D65" t="s">
+        <v>1246</v>
+      </c>
       <c r="F65">
         <v>65</v>
       </c>
@@ -5637,6 +5781,9 @@
       <c r="C66" t="s">
         <v>119</v>
       </c>
+      <c r="D66" t="s">
+        <v>1246</v>
+      </c>
       <c r="F66">
         <v>130</v>
       </c>
@@ -5654,6 +5801,9 @@
       <c r="C67" t="s">
         <v>119</v>
       </c>
+      <c r="D67" t="s">
+        <v>1246</v>
+      </c>
       <c r="F67">
         <v>130</v>
       </c>
@@ -5671,6 +5821,9 @@
       <c r="C68" t="s">
         <v>119</v>
       </c>
+      <c r="D68" t="s">
+        <v>1246</v>
+      </c>
       <c r="F68">
         <v>130</v>
       </c>
@@ -5688,6 +5841,9 @@
       <c r="C69" t="s">
         <v>119</v>
       </c>
+      <c r="D69" t="s">
+        <v>1246</v>
+      </c>
       <c r="F69">
         <v>130</v>
       </c>
@@ -5705,6 +5861,9 @@
       <c r="C70" t="s">
         <v>119</v>
       </c>
+      <c r="D70" t="s">
+        <v>1246</v>
+      </c>
       <c r="F70">
         <v>130</v>
       </c>
@@ -5722,6 +5881,9 @@
       <c r="C71" t="s">
         <v>119</v>
       </c>
+      <c r="D71" t="s">
+        <v>1246</v>
+      </c>
       <c r="F71">
         <v>130</v>
       </c>
@@ -5739,6 +5901,9 @@
       <c r="C72" t="s">
         <v>119</v>
       </c>
+      <c r="D72" t="s">
+        <v>1246</v>
+      </c>
       <c r="F72">
         <v>130</v>
       </c>
@@ -5756,6 +5921,9 @@
       <c r="C73" t="s">
         <v>119</v>
       </c>
+      <c r="D73" t="s">
+        <v>1246</v>
+      </c>
       <c r="F73">
         <v>130</v>
       </c>
@@ -5773,6 +5941,9 @@
       <c r="C74" t="s">
         <v>119</v>
       </c>
+      <c r="D74" t="s">
+        <v>1246</v>
+      </c>
       <c r="F74">
         <v>130</v>
       </c>
@@ -5790,6 +5961,9 @@
       <c r="C75" t="s">
         <v>119</v>
       </c>
+      <c r="D75" t="s">
+        <v>1246</v>
+      </c>
       <c r="F75">
         <v>130</v>
       </c>
@@ -5807,6 +5981,9 @@
       <c r="C76" t="s">
         <v>119</v>
       </c>
+      <c r="D76" t="s">
+        <v>1246</v>
+      </c>
       <c r="F76">
         <v>130</v>
       </c>
@@ -5824,6 +6001,9 @@
       <c r="C77" t="s">
         <v>119</v>
       </c>
+      <c r="D77" t="s">
+        <v>1246</v>
+      </c>
       <c r="F77">
         <v>130</v>
       </c>
@@ -5841,6 +6021,9 @@
       <c r="C78" t="s">
         <v>119</v>
       </c>
+      <c r="D78" t="s">
+        <v>1246</v>
+      </c>
       <c r="F78">
         <v>130</v>
       </c>
@@ -5858,6 +6041,9 @@
       <c r="C79" t="s">
         <v>119</v>
       </c>
+      <c r="D79" t="s">
+        <v>1246</v>
+      </c>
       <c r="F79">
         <v>130</v>
       </c>
@@ -5875,6 +6061,9 @@
       <c r="C80" t="s">
         <v>119</v>
       </c>
+      <c r="D80" t="s">
+        <v>1246</v>
+      </c>
       <c r="F80">
         <v>130</v>
       </c>
@@ -5892,6 +6081,9 @@
       <c r="C81" t="s">
         <v>119</v>
       </c>
+      <c r="D81" t="s">
+        <v>1246</v>
+      </c>
       <c r="F81">
         <v>130</v>
       </c>
@@ -5909,6 +6101,9 @@
       <c r="C82" t="s">
         <v>119</v>
       </c>
+      <c r="D82" t="s">
+        <v>1246</v>
+      </c>
       <c r="F82">
         <v>130</v>
       </c>
@@ -5926,6 +6121,9 @@
       <c r="C83" t="s">
         <v>119</v>
       </c>
+      <c r="D83" t="s">
+        <v>1246</v>
+      </c>
       <c r="F83">
         <v>130</v>
       </c>
@@ -5946,6 +6144,9 @@
       <c r="C84" t="s">
         <v>119</v>
       </c>
+      <c r="D84" t="s">
+        <v>1246</v>
+      </c>
       <c r="F84">
         <v>130</v>
       </c>
@@ -5963,6 +6164,9 @@
       <c r="C85" t="s">
         <v>119</v>
       </c>
+      <c r="D85" t="s">
+        <v>1246</v>
+      </c>
       <c r="F85">
         <v>130</v>
       </c>
@@ -5980,6 +6184,9 @@
       <c r="C86" t="s">
         <v>119</v>
       </c>
+      <c r="D86" t="s">
+        <v>1246</v>
+      </c>
       <c r="F86">
         <v>130</v>
       </c>
@@ -5997,6 +6204,9 @@
       <c r="C87" t="s">
         <v>119</v>
       </c>
+      <c r="D87" t="s">
+        <v>1246</v>
+      </c>
       <c r="F87">
         <v>130</v>
       </c>
@@ -6014,6 +6224,9 @@
       <c r="C88" t="s">
         <v>119</v>
       </c>
+      <c r="D88" t="s">
+        <v>1246</v>
+      </c>
       <c r="F88">
         <v>130</v>
       </c>
@@ -6031,6 +6244,9 @@
       <c r="C89" t="s">
         <v>119</v>
       </c>
+      <c r="D89" t="s">
+        <v>1246</v>
+      </c>
       <c r="F89">
         <v>130</v>
       </c>
@@ -6048,6 +6264,9 @@
       <c r="C90" t="s">
         <v>119</v>
       </c>
+      <c r="D90" t="s">
+        <v>1246</v>
+      </c>
       <c r="F90">
         <v>130</v>
       </c>
@@ -6065,6 +6284,9 @@
       <c r="C91" t="s">
         <v>119</v>
       </c>
+      <c r="D91" t="s">
+        <v>1246</v>
+      </c>
       <c r="F91">
         <v>130</v>
       </c>
@@ -6085,6 +6307,9 @@
       <c r="C92" t="s">
         <v>119</v>
       </c>
+      <c r="D92" t="s">
+        <v>1246</v>
+      </c>
       <c r="F92">
         <v>130</v>
       </c>
@@ -6102,6 +6327,9 @@
       <c r="C93" t="s">
         <v>119</v>
       </c>
+      <c r="D93" t="s">
+        <v>1246</v>
+      </c>
       <c r="F93">
         <v>130</v>
       </c>
@@ -6119,6 +6347,9 @@
       <c r="C94" t="s">
         <v>119</v>
       </c>
+      <c r="D94" t="s">
+        <v>1246</v>
+      </c>
       <c r="F94">
         <v>130</v>
       </c>
@@ -6136,6 +6367,9 @@
       <c r="C95" t="s">
         <v>119</v>
       </c>
+      <c r="D95" t="s">
+        <v>1246</v>
+      </c>
       <c r="F95">
         <v>130</v>
       </c>
@@ -6153,6 +6387,9 @@
       <c r="C96" t="s">
         <v>119</v>
       </c>
+      <c r="D96" t="s">
+        <v>1246</v>
+      </c>
       <c r="F96">
         <v>130</v>
       </c>
@@ -6170,6 +6407,9 @@
       <c r="C97" t="s">
         <v>119</v>
       </c>
+      <c r="D97" t="s">
+        <v>1246</v>
+      </c>
       <c r="F97">
         <v>130</v>
       </c>
@@ -6187,6 +6427,9 @@
       <c r="C98" t="s">
         <v>119</v>
       </c>
+      <c r="D98" t="s">
+        <v>1246</v>
+      </c>
       <c r="F98">
         <v>130</v>
       </c>
@@ -6204,6 +6447,9 @@
       <c r="C99" t="s">
         <v>119</v>
       </c>
+      <c r="D99" t="s">
+        <v>1246</v>
+      </c>
       <c r="F99">
         <v>130</v>
       </c>
@@ -6221,6 +6467,9 @@
       <c r="C100" t="s">
         <v>119</v>
       </c>
+      <c r="D100" t="s">
+        <v>1246</v>
+      </c>
       <c r="F100">
         <v>130</v>
       </c>
@@ -6238,6 +6487,9 @@
       <c r="C101" t="s">
         <v>119</v>
       </c>
+      <c r="D101" t="s">
+        <v>1246</v>
+      </c>
       <c r="F101">
         <v>130</v>
       </c>
@@ -6255,6 +6507,9 @@
       <c r="C102" t="s">
         <v>119</v>
       </c>
+      <c r="D102" t="s">
+        <v>1246</v>
+      </c>
       <c r="F102">
         <v>130</v>
       </c>
@@ -6272,6 +6527,9 @@
       <c r="C103" t="s">
         <v>119</v>
       </c>
+      <c r="D103" t="s">
+        <v>1246</v>
+      </c>
       <c r="F103">
         <v>130</v>
       </c>
@@ -6289,6 +6547,9 @@
       <c r="C104" t="s">
         <v>119</v>
       </c>
+      <c r="D104" t="s">
+        <v>1246</v>
+      </c>
       <c r="F104">
         <v>130</v>
       </c>
@@ -6306,6 +6567,9 @@
       <c r="C105" t="s">
         <v>119</v>
       </c>
+      <c r="D105" t="s">
+        <v>1246</v>
+      </c>
       <c r="F105">
         <v>130</v>
       </c>
@@ -6323,6 +6587,9 @@
       <c r="C106" t="s">
         <v>119</v>
       </c>
+      <c r="D106" t="s">
+        <v>1246</v>
+      </c>
       <c r="F106">
         <v>130</v>
       </c>
@@ -6340,6 +6607,9 @@
       <c r="C107" t="s">
         <v>119</v>
       </c>
+      <c r="D107" t="s">
+        <v>1246</v>
+      </c>
       <c r="F107">
         <v>130</v>
       </c>
@@ -6357,6 +6627,9 @@
       <c r="C108" t="s">
         <v>119</v>
       </c>
+      <c r="D108" t="s">
+        <v>1246</v>
+      </c>
       <c r="F108">
         <v>130</v>
       </c>
@@ -6374,6 +6647,9 @@
       <c r="C109" t="s">
         <v>119</v>
       </c>
+      <c r="D109" t="s">
+        <v>1246</v>
+      </c>
       <c r="F109">
         <v>130</v>
       </c>
@@ -6391,6 +6667,9 @@
       <c r="C110" t="s">
         <v>119</v>
       </c>
+      <c r="D110" t="s">
+        <v>1246</v>
+      </c>
       <c r="F110">
         <v>130</v>
       </c>
@@ -6408,6 +6687,9 @@
       <c r="C111" t="s">
         <v>119</v>
       </c>
+      <c r="D111" t="s">
+        <v>1246</v>
+      </c>
       <c r="F111">
         <v>130</v>
       </c>
@@ -6424,6 +6706,9 @@
       </c>
       <c r="C112" t="s">
         <v>119</v>
+      </c>
+      <c r="D112" t="s">
+        <v>1246</v>
       </c>
       <c r="F112">
         <v>130</v>

</xml_diff>

<commit_message>
updated core measurement records
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203CCC60-4059-403F-B800-2C9CDCEBFD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C462BF31-6879-4CB1-8734-6820047F4371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4024" uniqueCount="1257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4030" uniqueCount="1257">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -11323,6 +11323,15 @@
       <c r="C10" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D10" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E10" s="6">
+        <v>46266</v>
+      </c>
+      <c r="F10">
+        <v>94</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -11334,6 +11343,15 @@
       <c r="C11" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D11" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E11" s="6">
+        <v>46266</v>
+      </c>
+      <c r="F11">
+        <v>116</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -11345,6 +11363,15 @@
       <c r="C12" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D12" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E12" s="6">
+        <v>46266</v>
+      </c>
+      <c r="F12">
+        <v>130</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -11356,6 +11383,15 @@
       <c r="C13" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D13" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E13" s="6">
+        <v>46266</v>
+      </c>
+      <c r="F13">
+        <v>95</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -11367,6 +11403,15 @@
       <c r="C14" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D14" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E14" s="6">
+        <v>46267</v>
+      </c>
+      <c r="F14">
+        <v>130</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
@@ -11377,6 +11422,15 @@
       </c>
       <c r="C15" s="2" t="s">
         <v>232</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E15" s="6">
+        <v>46267</v>
+      </c>
+      <c r="F15">
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
core measurement records updated
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C462BF31-6879-4CB1-8734-6820047F4371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63794CB0-A8E9-492C-A945-D8D4C30346FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4030" uniqueCount="1257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4035" uniqueCount="1257">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -11443,6 +11443,15 @@
       <c r="C16" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D16" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E16" s="6">
+        <v>46268</v>
+      </c>
+      <c r="F16">
+        <v>113</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -11454,6 +11463,15 @@
       <c r="C17" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D17" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E17" s="6">
+        <v>46268</v>
+      </c>
+      <c r="F17">
+        <v>98</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
@@ -11465,6 +11483,15 @@
       <c r="C18" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D18" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E18" s="6">
+        <v>46268</v>
+      </c>
+      <c r="F18">
+        <v>130</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
@@ -11476,6 +11503,15 @@
       <c r="C19" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D19" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E19" s="6">
+        <v>46268</v>
+      </c>
+      <c r="F19">
+        <v>130</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
@@ -11486,6 +11522,15 @@
       </c>
       <c r="C20" s="2" t="s">
         <v>232</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E20" s="6">
+        <v>46268</v>
+      </c>
+      <c r="F20">
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>